<commit_message>
Correct coordinates for 5 flagged sites
Traðarholt: 63.5095, -19.6291 (was 65.89, -21.17)
Eyrarteigur: 65.1042, -14.6083 (was 65.06, -14.58)
Berufjörður: 64.7567, -14.4302 (was 65.54, -22.11)
Granagil/Skaftártunga: 63.7754, -18.4934 (was 63.08, -18.05)
Glaumbær: 65.7504, -17.4163 (was 65.70, -17.05)
Coord_flag cleared for all five; R map picks up changes from CSV.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/draftsNew/horse_sites_wgs84.xlsx
+++ b/draftsNew/horse_sites_wgs84.xlsx
@@ -1024,126 +1024,118 @@
       <c r="O9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Traðarholt, Stokkseyrarhreppi</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>THS</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Already permitted</t>
         </is>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Þjms. 1841 (IceEq15); Þjms. 1844 (IceEq16), Þjms. 1853</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>&lt; 1000</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>settlement</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Settlement (870–1100 CE)</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>&lt; 1000</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>settlement</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Settlement (870–1100 CE)</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Árnessýsla</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Suðurland</t>
         </is>
       </c>
-      <c r="K10" s="3" t="n">
-        <v>65.894886</v>
-      </c>
-      <c r="L10" s="3" t="n">
-        <v>-21.173493</v>
-      </c>
-      <c r="M10" s="3" t="inlineStr">
-        <is>
-          <t>ISN93→WGS84</t>
-        </is>
-      </c>
-      <c r="N10" s="3" t="inlineStr">
-        <is>
-          <t>ISN93 coords place site in north; Traðarholt is in Árnessýsla (south); Coord outside expected range for Árnessýsla (expected lat 63.5–64.6, lon -22.5–-18.5)</t>
-        </is>
-      </c>
-      <c r="O10" s="3" t="inlineStr"/>
+      <c r="K10" s="2" t="n">
+        <v>63.5095</v>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>-19.629139</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>corrected DMS</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Eyrarteigur (Þórisá)</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr"/>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Already permitted</t>
         </is>
       </c>
-      <c r="D11" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="D11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>Þjms. 1995-358 (IceEq7)</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>&lt; 1000</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>settlement</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>Settlement (870–1100 CE)</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr"/>
-      <c r="K11" s="3" t="n">
-        <v>65.060194</v>
-      </c>
-      <c r="L11" s="3" t="n">
-        <v>-14.578528</v>
-      </c>
-      <c r="M11" s="3" t="inlineStr">
-        <is>
-          <t>DMS→WGS84</t>
-        </is>
-      </c>
-      <c r="N11" s="3" t="inlineStr">
-        <is>
-          <t>Þórisá is in south Iceland; lon=-14.6 places this in east Iceland</t>
-        </is>
-      </c>
-      <c r="O11" s="3" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>&lt; 1000</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>settlement</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Settlement (870–1100 CE)</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="n">
+        <v>65.104167</v>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>-14.608333</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>corrected DMS</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1319,59 +1311,55 @@
       <c r="O14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Berufjörður</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr"/>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Already permitted</t>
         </is>
       </c>
-      <c r="D15" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="D15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>Þjms. 4489 (IceEq2)</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>&lt; 1000</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>settlement</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Settlement (870–1100 CE)</t>
-        </is>
-      </c>
-      <c r="I15" s="3" t="inlineStr"/>
-      <c r="J15" s="3" t="inlineStr"/>
-      <c r="K15" s="3" t="n">
-        <v>65.538</v>
-      </c>
-      <c r="L15" s="3" t="n">
-        <v>-22.11</v>
-      </c>
-      <c r="M15" s="3" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="N15" s="3" t="inlineStr">
-        <is>
-          <t>Berufjörður is in Eastfjords (~64.8°N, -14.2°W); coords look wrong</t>
-        </is>
-      </c>
-      <c r="O15" s="3" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>&lt; 1000</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>settlement</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Settlement (870–1100 CE)</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="n">
+        <v>64.7567</v>
+      </c>
+      <c r="L15" s="2" t="n">
+        <v>-14.4302</v>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>corrected decimal</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2210,67 +2198,63 @@
       <c r="O31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Granagil hjá Búlandi í Skaftártunguhreppi</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>GGS</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>In new request</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="n">
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>In new request</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
         <is>
           <t>Þjms. 11526; Þjms. 6419b</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>&lt; 1000</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>settlement</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>Settlement (870–1100 CE)</t>
-        </is>
-      </c>
-      <c r="I32" s="3" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>&lt; 1000</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>settlement</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>Settlement (870–1100 CE)</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
         <is>
           <t>V-Skaftafellssýsla</t>
         </is>
       </c>
-      <c r="J32" s="3" t="inlineStr"/>
-      <c r="K32" s="3" t="n">
-        <v>63.08</v>
-      </c>
-      <c r="L32" s="3" t="n">
-        <v>-18.05</v>
-      </c>
-      <c r="M32" s="3" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="N32" s="3" t="inlineStr">
-        <is>
-          <t>Coord outside expected range for V-Skaftafellssýsla (expected lat 63.3–64.3, lon -19.5–-17.0)</t>
-        </is>
-      </c>
-      <c r="O32" s="3" t="inlineStr"/>
+      <c r="J32" s="4" t="inlineStr"/>
+      <c r="K32" s="4" t="n">
+        <v>63.775444</v>
+      </c>
+      <c r="L32" s="4" t="n">
+        <v>-18.493417</v>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>corrected DMS</t>
+        </is>
+      </c>
+      <c r="N32" s="4" t="inlineStr"/>
+      <c r="O32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -3115,67 +3099,63 @@
       <c r="O46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>Glaumbær</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>GBR</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>In new request</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="n">
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>In new request</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E47" s="4" t="inlineStr">
         <is>
           <t>Þjms. 6918; Þjms. 6921; Þjms. 6933</t>
         </is>
       </c>
-      <c r="F47" s="3" t="inlineStr">
-        <is>
-          <t>&lt; 1000</t>
-        </is>
-      </c>
-      <c r="G47" s="3" t="inlineStr">
-        <is>
-          <t>settlement</t>
-        </is>
-      </c>
-      <c r="H47" s="3" t="inlineStr">
-        <is>
-          <t>Settlement (870–1100 CE)</t>
-        </is>
-      </c>
-      <c r="I47" s="3" t="inlineStr">
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>&lt; 1000</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>settlement</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>Settlement (870–1100 CE)</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
         <is>
           <t>S-Þingeyjarsýsla</t>
         </is>
       </c>
-      <c r="J47" s="3" t="inlineStr"/>
-      <c r="K47" s="3" t="n">
-        <v>65.7</v>
-      </c>
-      <c r="L47" s="3" t="n">
-        <v>-17.05</v>
-      </c>
-      <c r="M47" s="3" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="N47" s="3" t="inlineStr">
-        <is>
-          <t>Famous Glaumbær (Skagafjörður) should be ~65.6°N, -19.5°W</t>
-        </is>
-      </c>
-      <c r="O47" s="3" t="inlineStr"/>
+      <c r="J47" s="4" t="inlineStr"/>
+      <c r="K47" s="4" t="n">
+        <v>65.750389</v>
+      </c>
+      <c r="L47" s="4" t="n">
+        <v>-17.416333</v>
+      </c>
+      <c r="M47" s="4" t="inlineStr">
+        <is>
+          <t>corrected DMS</t>
+        </is>
+      </c>
+      <c r="N47" s="4" t="inlineStr"/>
+      <c r="O47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Fix map R script: coord_ok bug, add labels for overlapping sites, correct Granagil and Traðarholt coordinates
- Fix 'object coord_ok not found' error by using base-R subsetting instead of dplyr filter()
- Add ggrepel labels for sites that overlap on map (Alþingisreitur, Tjarnargata, Vatnsdalur, Staðartunga)
- Update Granagil (63.7857, -18.5093) and Traðarholt (63.8415, -21.0034) coordinates in CSV and xlsx

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/draftsNew/horse_sites_wgs84.xlsx
+++ b/draftsNew/horse_sites_wgs84.xlsx
@@ -1073,10 +1073,10 @@
         </is>
       </c>
       <c r="K10" s="2" t="n">
-        <v>63.5095</v>
+        <v>63.84148</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>-19.629139</v>
+        <v>-21.00337</v>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
@@ -2243,14 +2243,14 @@
       </c>
       <c r="J32" s="4" t="inlineStr"/>
       <c r="K32" s="4" t="n">
-        <v>63.775444</v>
+        <v>63.7857</v>
       </c>
       <c r="L32" s="4" t="n">
-        <v>-18.493417</v>
+        <v>-18.509333</v>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>corrected DMS</t>
+          <t>corrected decimal-minutes</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Update coordinates for Granagil and Traðarholt
Granagil hjá Búlandi: 63.783245, -18.583696
Traðarholt, Stokkseyrarhreppi: 63.837994, -21.015610

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/draftsNew/horse_sites_wgs84.xlsx
+++ b/draftsNew/horse_sites_wgs84.xlsx
@@ -1073,10 +1073,10 @@
         </is>
       </c>
       <c r="K10" s="2" t="n">
-        <v>63.84148</v>
+        <v>63.837994</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>-21.00337</v>
+        <v>-21.01561</v>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
@@ -2243,10 +2243,10 @@
       </c>
       <c r="J32" s="4" t="inlineStr"/>
       <c r="K32" s="4" t="n">
-        <v>63.7857</v>
+        <v>63.783245</v>
       </c>
       <c r="L32" s="4" t="n">
-        <v>-18.509333</v>
+        <v>-18.583696</v>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Remove duplicate Vatnsdalur and Staðartunga sites; merge into single rows
- Vatnsdalur við Patreksfjörð removed; merged into Vatnsdalur í Patreksfirði (N=2, both museum numbers)
- Staðartunga í Hörgárdal HSE row removed; merged into STH row (N=2, Þjms. 11716 + Þjms. 11435)
- R script: remove now-redundant labels for those sites

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/draftsNew/horse_sites_wgs84.xlsx
+++ b/draftsNew/horse_sites_wgs84.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O71"/>
+  <dimension ref="A1:O69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -2039,14 +2039,10 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Vatnsdalur við Patreksfjörð</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>VDP</t>
-        </is>
-      </c>
+          <t>Þórðarholt</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr"/>
       <c r="C29" s="4" t="inlineStr">
         <is>
           <t>In new request</t>
@@ -2057,7 +2053,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>1968-510</t>
+          <t>Þjms. 12562</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -2075,21 +2071,17 @@
           <t>Settlement (870–1100 CE)</t>
         </is>
       </c>
-      <c r="I29" s="4" t="inlineStr">
-        <is>
-          <t>Barðastrandasýsla</t>
-        </is>
-      </c>
+      <c r="I29" s="4" t="inlineStr"/>
       <c r="J29" s="4" t="inlineStr"/>
       <c r="K29" s="4" t="n">
-        <v>65.56999999999999</v>
+        <v>64.11666700000001</v>
       </c>
       <c r="L29" s="4" t="n">
-        <v>-24.07</v>
+        <v>-19.75</v>
       </c>
       <c r="M29" s="4" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>DMS→WGS84</t>
         </is>
       </c>
       <c r="N29" s="4" t="inlineStr"/>
@@ -2098,7 +2090,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Þórðarholt</t>
+          <t>Þóreyjarnúpur</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr"/>
@@ -2112,7 +2104,7 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 12562</t>
+          <t>Þjms. 10435a</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -2133,10 +2125,10 @@
       <c r="I30" s="4" t="inlineStr"/>
       <c r="J30" s="4" t="inlineStr"/>
       <c r="K30" s="4" t="n">
-        <v>64.11666700000001</v>
+        <v>65.37925</v>
       </c>
       <c r="L30" s="4" t="n">
-        <v>-19.75</v>
+        <v>-20.727806</v>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
@@ -2149,21 +2141,25 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Þóreyjarnúpur</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr"/>
+          <t>Granagil hjá Búlandi í Skaftártunguhreppi</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>GGS</t>
+        </is>
+      </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
           <t>In new request</t>
         </is>
       </c>
       <c r="D31" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 10435a</t>
+          <t>Þjms. 11526; Þjms. 6419b</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -2181,17 +2177,21 @@
           <t>Settlement (870–1100 CE)</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr"/>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>V-Skaftafellssýsla</t>
+        </is>
+      </c>
       <c r="J31" s="4" t="inlineStr"/>
       <c r="K31" s="4" t="n">
-        <v>65.37925</v>
+        <v>63.783245</v>
       </c>
       <c r="L31" s="4" t="n">
-        <v>-20.727806</v>
+        <v>-18.583696</v>
       </c>
       <c r="M31" s="4" t="inlineStr">
         <is>
-          <t>DMS→WGS84</t>
+          <t>corrected decimal-minutes</t>
         </is>
       </c>
       <c r="N31" s="4" t="inlineStr"/>
@@ -2200,12 +2200,12 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Granagil hjá Búlandi í Skaftártunguhreppi</t>
+          <t>Kápa  á Almenningum</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>GGS</t>
+          <t>KVE</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -2214,11 +2214,11 @@
         </is>
       </c>
       <c r="D32" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 11526; Þjms. 6419b</t>
+          <t>Nokkrar hrossatennur (2434)</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -2238,19 +2238,19 @@
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>V-Skaftafellssýsla</t>
+          <t>Rangárvallarsýsla</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr"/>
       <c r="K32" s="4" t="n">
-        <v>63.783245</v>
+        <v>63.5264</v>
       </c>
       <c r="L32" s="4" t="n">
-        <v>-18.583696</v>
+        <v>-19.4733</v>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>corrected decimal-minutes</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr"/>
@@ -2259,12 +2259,12 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Kápa  á Almenningum</t>
+          <t>Hrífunes, Skaftártunga</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>KVE</t>
+          <t>HRS</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Nokkrar hrossatennur (2434)</t>
+          <t>1958-133</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -2297,15 +2297,15 @@
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Rangárvallarsýsla</t>
+          <t>V-Skaftafellssýsla</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr"/>
       <c r="K33" s="4" t="n">
-        <v>63.5264</v>
+        <v>63.6957</v>
       </c>
       <c r="L33" s="4" t="n">
-        <v>-19.4733</v>
+        <v>-18.3771</v>
       </c>
       <c r="M33" s="4" t="inlineStr">
         <is>
@@ -2318,12 +2318,12 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Hrífunes, Skaftártunga</t>
+          <t>Stóri-Moshvoll, Hvolhreppur</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>HRS</t>
+          <t>SMH</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>1958-133</t>
+          <t>1912 hrossabein</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -2356,15 +2356,15 @@
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>V-Skaftafellssýsla</t>
+          <t>Rangárvallarsýsla</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr"/>
       <c r="K34" s="4" t="n">
-        <v>63.6957</v>
+        <v>63.74</v>
       </c>
       <c r="L34" s="4" t="n">
-        <v>-18.3771</v>
+        <v>-20.204</v>
       </c>
       <c r="M34" s="4" t="inlineStr">
         <is>
@@ -2377,12 +2377,12 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Stóri-Moshvoll, Hvolhreppur</t>
+          <t>Mörk í Landssveit</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>SMH</t>
+          <t>MKL</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>1912 hrossabein</t>
+          <t>Þjms. 11920</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -2418,12 +2418,16 @@
           <t>Rangárvallarsýsla</t>
         </is>
       </c>
-      <c r="J35" s="4" t="inlineStr"/>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>Suðurland</t>
+        </is>
+      </c>
       <c r="K35" s="4" t="n">
-        <v>63.74</v>
+        <v>64.03</v>
       </c>
       <c r="L35" s="4" t="n">
-        <v>-20.204</v>
+        <v>-20.02</v>
       </c>
       <c r="M35" s="4" t="inlineStr">
         <is>
@@ -2436,12 +2440,12 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Mörk í Landssveit</t>
+          <t>Hólaskógur, Gnjúpverjahreppur</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>MKL</t>
+          <t>ÞHS</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -2454,7 +2458,7 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 11920</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -2477,16 +2481,12 @@
           <t>Rangárvallarsýsla</t>
         </is>
       </c>
-      <c r="J36" s="4" t="inlineStr">
-        <is>
-          <t>Suðurland</t>
-        </is>
-      </c>
+      <c r="J36" s="4" t="inlineStr"/>
       <c r="K36" s="4" t="n">
-        <v>64.03</v>
+        <v>64.1275</v>
       </c>
       <c r="L36" s="4" t="n">
-        <v>-20.02</v>
+        <v>-19.75</v>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
@@ -2499,53 +2499,47 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Hólaskógur, Gnjúpverjahreppur</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>ÞHS</t>
-        </is>
-      </c>
+          <t>Alþingisreitur</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr"/>
       <c r="C37" s="4" t="inlineStr">
         <is>
           <t>In new request</t>
         </is>
       </c>
-      <c r="D37" s="4" t="n">
-        <v>1</v>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>4+</t>
+        </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>K-5-M-6</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>&lt; 1000</t>
+          <t>1600–1800</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>settlement</t>
+          <t>post-settlement</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>Settlement (870–1100 CE)</t>
-        </is>
-      </c>
-      <c r="I37" s="4" t="inlineStr">
-        <is>
-          <t>Rangárvallarsýsla</t>
-        </is>
-      </c>
+          <t>Post-medieval (1100–1900 CE)</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr"/>
       <c r="J37" s="4" t="inlineStr"/>
       <c r="K37" s="4" t="n">
-        <v>64.1275</v>
+        <v>64.15000000000001</v>
       </c>
       <c r="L37" s="4" t="n">
-        <v>-19.75</v>
+        <v>-21.94</v>
       </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
@@ -2558,10 +2552,14 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Alþingisreitur</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr"/>
+          <t>Skriðuklaustur í Fljótsdal</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>SKR</t>
+        </is>
+      </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
           <t>In new request</t>
@@ -2569,17 +2567,17 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>4+</t>
+          <t>30+</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>K-5-M-6</t>
+          <t>SKR (many boxes)</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>1600–1800</t>
+          <t>1450–1800</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -2595,10 +2593,10 @@
       <c r="I38" s="4" t="inlineStr"/>
       <c r="J38" s="4" t="inlineStr"/>
       <c r="K38" s="4" t="n">
-        <v>64.15000000000001</v>
+        <v>65.04000000000001</v>
       </c>
       <c r="L38" s="4" t="n">
-        <v>-21.94</v>
+        <v>-14.95</v>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
@@ -2611,12 +2609,12 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Skriðuklaustur í Fljótsdal</t>
+          <t>Hrollaugsstaðir</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>SKR</t>
+          <t>HLS</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -2624,38 +2622,40 @@
           <t>In new request</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>30+</t>
-        </is>
+      <c r="D39" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>SKR (many boxes)</t>
+          <t>Þjms. 15227b</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>1450–1800</t>
+          <t>&lt; 1000</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>post-settlement</t>
+          <t>settlement</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Post-medieval (1100–1900 CE)</t>
-        </is>
-      </c>
-      <c r="I39" s="4" t="inlineStr"/>
+          <t>Settlement (870–1100 CE)</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>N-Múlasýsla</t>
+        </is>
+      </c>
       <c r="J39" s="4" t="inlineStr"/>
       <c r="K39" s="4" t="n">
-        <v>65.04000000000001</v>
+        <v>65.11879999999999</v>
       </c>
       <c r="L39" s="4" t="n">
-        <v>-14.95</v>
+        <v>-15.0146</v>
       </c>
       <c r="M39" s="4" t="inlineStr">
         <is>
@@ -2668,12 +2668,12 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>Hrollaugsstaðir</t>
+          <t>Fjörður í Seyðisfirði</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>HLS</t>
+          <t>FJO</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -2686,7 +2686,7 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 15227b</t>
+          <t>15229</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
@@ -2706,15 +2706,19 @@
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>N-Múlasýsla</t>
-        </is>
-      </c>
-      <c r="J40" s="4" t="inlineStr"/>
+          <t>Seyðisfjarðarsýsla</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>Austurland</t>
+        </is>
+      </c>
       <c r="K40" s="4" t="n">
-        <v>65.11879999999999</v>
+        <v>65.29000000000001</v>
       </c>
       <c r="L40" s="4" t="n">
-        <v>-15.0146</v>
+        <v>-13.76</v>
       </c>
       <c r="M40" s="4" t="inlineStr">
         <is>
@@ -2722,17 +2726,21 @@
         </is>
       </c>
       <c r="N40" s="4" t="inlineStr"/>
-      <c r="O40" s="4" t="inlineStr"/>
+      <c r="O40" s="4" t="inlineStr">
+        <is>
+          <t>Horse mentioned in human sample notes but no corresponding horse entry found in Horses.docx from Joe</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>Fjörður í Seyðisfirði</t>
+          <t>Reykjasel, Jökuldalshreppi</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>FJO</t>
+          <t>RSJ</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -2745,7 +2753,7 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>15229</t>
+          <t>Þjms. 4867</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
@@ -2765,19 +2773,15 @@
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Seyðisfjarðarsýsla</t>
-        </is>
-      </c>
-      <c r="J41" s="4" t="inlineStr">
-        <is>
-          <t>Austurland</t>
-        </is>
-      </c>
+          <t>N-Múlasýsla</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr"/>
       <c r="K41" s="4" t="n">
-        <v>65.29000000000001</v>
+        <v>65.3092</v>
       </c>
       <c r="L41" s="4" t="n">
-        <v>-13.76</v>
+        <v>-15.1638</v>
       </c>
       <c r="M41" s="4" t="inlineStr">
         <is>
@@ -2785,21 +2789,17 @@
         </is>
       </c>
       <c r="N41" s="4" t="inlineStr"/>
-      <c r="O41" s="4" t="inlineStr">
-        <is>
-          <t>Horse mentioned in human sample notes but no corresponding horse entry found in Horses.docx from Joe</t>
-        </is>
-      </c>
+      <c r="O41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Reykjasel, Jökuldalshreppi</t>
+          <t>Straumur í Tunguhreppi</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>RSJ</t>
+          <t>STT</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 4867</t>
+          <t>Þjoms. (in a box with artifacts)</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
@@ -2835,12 +2835,16 @@
           <t>N-Múlasýsla</t>
         </is>
       </c>
-      <c r="J42" s="4" t="inlineStr"/>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Austurland</t>
+        </is>
+      </c>
       <c r="K42" s="4" t="n">
-        <v>65.3092</v>
+        <v>65.44</v>
       </c>
       <c r="L42" s="4" t="n">
-        <v>-15.1638</v>
+        <v>-14.39</v>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
@@ -2848,17 +2852,21 @@
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr"/>
-      <c r="O42" s="4" t="inlineStr"/>
+      <c r="O42" s="4" t="inlineStr">
+        <is>
+          <t>Horse mentioned in human sample notes but no corresponding horse entry found in Horses.docx from Joe</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Straumur í Tunguhreppi</t>
+          <t>Ytri-Neslönd, Mývatnssveit</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>STT</t>
+          <t>YNM</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -2871,7 +2879,7 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>Þjoms. (in a box with artifacts)</t>
+          <t>1960-46</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
@@ -2891,19 +2899,15 @@
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>N-Múlasýsla</t>
-        </is>
-      </c>
-      <c r="J43" s="4" t="inlineStr">
-        <is>
-          <t>Austurland</t>
-        </is>
-      </c>
+          <t>S-Þingeyjarsýsla</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr"/>
       <c r="K43" s="4" t="n">
-        <v>65.44</v>
+        <v>65.62</v>
       </c>
       <c r="L43" s="4" t="n">
-        <v>-14.39</v>
+        <v>-17</v>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
@@ -2911,21 +2915,17 @@
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr"/>
-      <c r="O43" s="4" t="inlineStr">
-        <is>
-          <t>Horse mentioned in human sample notes but no corresponding horse entry found in Horses.docx from Joe</t>
-        </is>
-      </c>
+      <c r="O43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Ytri-Neslönd, Mývatnssveit</t>
+          <t>Staðartunga í Hörgárdal</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>YNM</t>
+          <t>STH</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -2934,11 +2934,11 @@
         </is>
       </c>
       <c r="D44" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>1960-46</t>
+          <t>Þjms. 11716; Þjms. 11435</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
@@ -2958,15 +2958,19 @@
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>S-Þingeyjarsýsla</t>
-        </is>
-      </c>
-      <c r="J44" s="4" t="inlineStr"/>
+          <t>Eyjafjarðarsýsla</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>Norðurland</t>
+        </is>
+      </c>
       <c r="K44" s="4" t="n">
-        <v>65.62</v>
+        <v>65.67</v>
       </c>
       <c r="L44" s="4" t="n">
-        <v>-17</v>
+        <v>-18.46</v>
       </c>
       <c r="M44" s="4" t="inlineStr">
         <is>
@@ -2979,12 +2983,12 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>Staðartunga í Hörgárdal</t>
+          <t>Glaumbær</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>HSE</t>
+          <t>GBR</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -2993,11 +2997,11 @@
         </is>
       </c>
       <c r="D45" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 11435</t>
+          <t>Þjms. 6918; Þjms. 6921; Þjms. 6933</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
@@ -3017,19 +3021,19 @@
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Eyjafjarðarsýsla</t>
+          <t>S-Þingeyjarsýsla</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr"/>
       <c r="K45" s="4" t="n">
-        <v>65.64</v>
+        <v>65.750389</v>
       </c>
       <c r="L45" s="4" t="n">
-        <v>-18.22</v>
+        <v>-17.416333</v>
       </c>
       <c r="M45" s="4" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>corrected DMS</t>
         </is>
       </c>
       <c r="N45" s="4" t="inlineStr"/>
@@ -3038,12 +3042,12 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Staðartunga í Hörgárdal</t>
+          <t>Hrafnsstaðir (í Kinn)</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>STH</t>
+          <t>HRK</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -3056,7 +3060,7 @@
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 11716</t>
+          <t>15234</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
@@ -3076,7 +3080,7 @@
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>Eyjafjarðarsýsla</t>
+          <t>S-Þingeyjarsýsla</t>
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr">
@@ -3085,10 +3089,10 @@
         </is>
       </c>
       <c r="K46" s="4" t="n">
-        <v>65.67</v>
+        <v>65.81</v>
       </c>
       <c r="L46" s="4" t="n">
-        <v>-18.46</v>
+        <v>-17.57</v>
       </c>
       <c r="M46" s="4" t="inlineStr">
         <is>
@@ -3096,17 +3100,21 @@
         </is>
       </c>
       <c r="N46" s="4" t="inlineStr"/>
-      <c r="O46" s="4" t="inlineStr"/>
+      <c r="O46" s="4" t="inlineStr">
+        <is>
+          <t>Horse mentioned in human sample notes but no corresponding horse entry found in Horses.docx from Joe</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>Glaumbær</t>
+          <t>Litlu-Núpar</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>GBR</t>
+          <t>NUA</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -3115,11 +3123,11 @@
         </is>
       </c>
       <c r="D47" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 6918; Þjms. 6921; Þjms. 6933</t>
+          <t>6948a/b</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -3139,33 +3147,41 @@
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>S-Þingeyjarsýsla</t>
-        </is>
-      </c>
-      <c r="J47" s="4" t="inlineStr"/>
+          <t>S-Þingeyjasýsla</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>Norðurland</t>
+        </is>
+      </c>
       <c r="K47" s="4" t="n">
-        <v>65.750389</v>
+        <v>65.95</v>
       </c>
       <c r="L47" s="4" t="n">
-        <v>-17.416333</v>
+        <v>-17.4</v>
       </c>
       <c r="M47" s="4" t="inlineStr">
         <is>
-          <t>corrected DMS</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="N47" s="4" t="inlineStr"/>
-      <c r="O47" s="4" t="inlineStr"/>
+      <c r="O47" s="4" t="inlineStr">
+        <is>
+          <t>Horse mentioned in human sample notes but no corresponding horse entry found in Horses.docx from Joe</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>Hrafnsstaðir (í Kinn)</t>
+          <t>Brimnes (Dalvík)</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>HRK</t>
+          <t>DAV</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -3174,11 +3190,11 @@
         </is>
       </c>
       <c r="D48" s="4" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>15234</t>
+          <t>Þjms. 5846 / Dys II (IceEq3); Þjms. 5856 / Dys XIII (IceEq4), Þjms. 6040; Þjms. 5849</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
@@ -3198,7 +3214,7 @@
       </c>
       <c r="I48" s="4" t="inlineStr">
         <is>
-          <t>S-Þingeyjarsýsla</t>
+          <t>Eyjafjarðarsýsla</t>
         </is>
       </c>
       <c r="J48" s="4" t="inlineStr">
@@ -3207,32 +3223,28 @@
         </is>
       </c>
       <c r="K48" s="4" t="n">
-        <v>65.81</v>
+        <v>65.97618799999999</v>
       </c>
       <c r="L48" s="4" t="n">
-        <v>-17.57</v>
+        <v>-18.530555</v>
       </c>
       <c r="M48" s="4" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>ISN93→WGS84</t>
         </is>
       </c>
       <c r="N48" s="4" t="inlineStr"/>
-      <c r="O48" s="4" t="inlineStr">
-        <is>
-          <t>Horse mentioned in human sample notes but no corresponding horse entry found in Horses.docx from Joe</t>
-        </is>
-      </c>
+      <c r="O48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Litlu-Núpar</t>
+          <t>Kolsholt í Flóa, Villingarholtshreppur</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>NUA</t>
+          <t>KHF</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -3245,7 +3257,7 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>6948a/b</t>
+          <t>Þjms. 1958:117</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
@@ -3265,41 +3277,33 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>S-Þingeyjasýsla</t>
-        </is>
-      </c>
-      <c r="J49" s="4" t="inlineStr">
-        <is>
-          <t>Norðurland</t>
-        </is>
-      </c>
+          <t>Árnessýsla</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="inlineStr"/>
       <c r="K49" s="4" t="n">
-        <v>65.95</v>
+        <v>63.872868</v>
       </c>
       <c r="L49" s="4" t="n">
-        <v>-17.4</v>
+        <v>-20.819098</v>
       </c>
       <c r="M49" s="4" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>ISN93→WGS84</t>
         </is>
       </c>
       <c r="N49" s="4" t="inlineStr"/>
-      <c r="O49" s="4" t="inlineStr">
-        <is>
-          <t>Horse mentioned in human sample notes but no corresponding horse entry found in Horses.docx from Joe</t>
-        </is>
-      </c>
+      <c r="O49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Brimnes (Dalvík)</t>
+          <t>Lækur í Hraungerðishreppi</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>DAV</t>
+          <t>LKH</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
@@ -3308,11 +3312,11 @@
         </is>
       </c>
       <c r="D50" s="4" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 5846 / Dys II (IceEq3); Þjms. 5856 / Dys XIII (IceEq4), Þjms. 6040; Þjms. 5849</t>
+          <t>1969-154</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
@@ -3332,19 +3336,19 @@
       </c>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>Eyjafjarðarsýsla</t>
+          <t>Árnessýsla</t>
         </is>
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>Norðurland</t>
+          <t>Suðurland</t>
         </is>
       </c>
       <c r="K50" s="4" t="n">
-        <v>65.97618799999999</v>
+        <v>63.918951</v>
       </c>
       <c r="L50" s="4" t="n">
-        <v>-18.530555</v>
+        <v>-20.877272</v>
       </c>
       <c r="M50" s="4" t="inlineStr">
         <is>
@@ -3357,12 +3361,12 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Kolsholt í Flóa, Villingarholtshreppur</t>
+          <t>Brandsstaðir í Blöndudal</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>KHF</t>
+          <t>BRB</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
@@ -3375,7 +3379,7 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 1958:117</t>
+          <t>1967-81/1996-269</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
@@ -3395,15 +3399,15 @@
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>Árnessýsla</t>
+          <t>A-Húnavatnssýsla</t>
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr"/>
       <c r="K51" s="4" t="n">
-        <v>63.872868</v>
+        <v>65.392449</v>
       </c>
       <c r="L51" s="4" t="n">
-        <v>-20.819098</v>
+        <v>-19.784325</v>
       </c>
       <c r="M51" s="4" t="inlineStr">
         <is>
@@ -3416,12 +3420,12 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>Lækur í Hraungerðishreppi</t>
+          <t>Öxnadalsheiði</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>LKH</t>
+          <t>OXH</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
@@ -3434,7 +3438,7 @@
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>1969-154</t>
+          <t>1962-209</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
@@ -3454,19 +3458,15 @@
       </c>
       <c r="I52" s="4" t="inlineStr">
         <is>
-          <t>Árnessýsla</t>
-        </is>
-      </c>
-      <c r="J52" s="4" t="inlineStr">
-        <is>
-          <t>Suðurland</t>
-        </is>
-      </c>
+          <t>Skagafjarðarsýsla</t>
+        </is>
+      </c>
+      <c r="J52" s="4" t="inlineStr"/>
       <c r="K52" s="4" t="n">
-        <v>63.918951</v>
+        <v>65.45168</v>
       </c>
       <c r="L52" s="4" t="n">
-        <v>-20.877272</v>
+        <v>-18.973369</v>
       </c>
       <c r="M52" s="4" t="inlineStr">
         <is>
@@ -3479,12 +3479,12 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>Brandsstaðir í Blöndudal</t>
+          <t>Elivogar/Langholt</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>BRB</t>
+          <t>EVS</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -3497,7 +3497,7 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>1967-81/1996-269</t>
+          <t>Þjms. 15690</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
@@ -3517,15 +3517,19 @@
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>A-Húnavatnssýsla</t>
-        </is>
-      </c>
-      <c r="J53" s="4" t="inlineStr"/>
+          <t>Skagafjarðarsýsla</t>
+        </is>
+      </c>
+      <c r="J53" s="4" t="inlineStr">
+        <is>
+          <t>Norðurland</t>
+        </is>
+      </c>
       <c r="K53" s="4" t="n">
-        <v>65.392449</v>
+        <v>65.568522</v>
       </c>
       <c r="L53" s="4" t="n">
-        <v>-19.784325</v>
+        <v>-19.563526</v>
       </c>
       <c r="M53" s="4" t="inlineStr">
         <is>
@@ -3538,12 +3542,12 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>Öxnadalsheiði</t>
+          <t>Sólheimar, Sæmundarhlíð</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>OXH</t>
+          <t>SHS</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -3556,7 +3560,7 @@
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>1962-209</t>
+          <t>Þjms. 15688</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
@@ -3581,10 +3585,10 @@
       </c>
       <c r="J54" s="4" t="inlineStr"/>
       <c r="K54" s="4" t="n">
-        <v>65.45168</v>
+        <v>65.597905</v>
       </c>
       <c r="L54" s="4" t="n">
-        <v>-18.973369</v>
+        <v>-19.585128</v>
       </c>
       <c r="M54" s="4" t="inlineStr">
         <is>
@@ -3597,12 +3601,12 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>Elivogar/Langholt</t>
+          <t>Vatnsdalur í Patreksfirði</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>EVS</t>
+          <t>VDP</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -3611,11 +3615,11 @@
         </is>
       </c>
       <c r="D55" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 15690</t>
+          <t>1964:136; 1968-510</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
@@ -3635,19 +3639,15 @@
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>Skagafjarðarsýsla</t>
-        </is>
-      </c>
-      <c r="J55" s="4" t="inlineStr">
-        <is>
-          <t>Norðurland</t>
-        </is>
-      </c>
+          <t>Barðastrandasýsla</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr"/>
       <c r="K55" s="4" t="n">
-        <v>65.568522</v>
+        <v>65.57238599999999</v>
       </c>
       <c r="L55" s="4" t="n">
-        <v>-19.563526</v>
+        <v>-24.061639</v>
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
@@ -3660,12 +3660,12 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>Sólheimar, Sæmundarhlíð</t>
+          <t>Sílastaðir, Glæsibæjarhreppi</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>SHS</t>
+          <t>SSG</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -3674,11 +3674,11 @@
         </is>
       </c>
       <c r="D56" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 15688</t>
+          <t>Þjms. 13702; Þjms. 13735</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
@@ -3698,15 +3698,19 @@
       </c>
       <c r="I56" s="4" t="inlineStr">
         <is>
-          <t>Skagafjarðarsýsla</t>
-        </is>
-      </c>
-      <c r="J56" s="4" t="inlineStr"/>
+          <t>Eyjafjarðarsýsla</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>Norðurland</t>
+        </is>
+      </c>
       <c r="K56" s="4" t="n">
-        <v>65.597905</v>
+        <v>65.72170300000001</v>
       </c>
       <c r="L56" s="4" t="n">
-        <v>-19.585128</v>
+        <v>-18.189824</v>
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
@@ -3719,12 +3723,12 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>Vatnsdalur í Patreksfirði</t>
+          <t>Brimnes, Viðvikurhreppur</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>VDP</t>
+          <t>BRV</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -3737,7 +3741,7 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>1964:136</t>
+          <t>Þjms.6040</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
@@ -3757,15 +3761,15 @@
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>Barðastrandasýsla</t>
+          <t>Skagafjarðarsýsla</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr"/>
       <c r="K57" s="4" t="n">
-        <v>65.57238599999999</v>
+        <v>65.777175</v>
       </c>
       <c r="L57" s="4" t="n">
-        <v>-24.061639</v>
+        <v>-19.34862</v>
       </c>
       <c r="M57" s="4" t="inlineStr">
         <is>
@@ -3778,12 +3782,12 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>Sílastaðir, Glæsibæjarhreppi</t>
+          <t>Grafargerði á Höfðaströnd</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>SSG</t>
+          <t>GGH</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -3792,11 +3796,11 @@
         </is>
       </c>
       <c r="D58" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 13702; Þjms. 13735</t>
+          <t>11685-b</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
@@ -3816,7 +3820,7 @@
       </c>
       <c r="I58" s="4" t="inlineStr">
         <is>
-          <t>Eyjafjarðarsýsla</t>
+          <t>Skagafjarðarsýsla</t>
         </is>
       </c>
       <c r="J58" s="4" t="inlineStr">
@@ -3825,10 +3829,10 @@
         </is>
       </c>
       <c r="K58" s="4" t="n">
-        <v>65.72170300000001</v>
+        <v>65.881074</v>
       </c>
       <c r="L58" s="4" t="n">
-        <v>-18.189824</v>
+        <v>-19.392373</v>
       </c>
       <c r="M58" s="4" t="inlineStr">
         <is>
@@ -3836,17 +3840,21 @@
         </is>
       </c>
       <c r="N58" s="4" t="inlineStr"/>
-      <c r="O58" s="4" t="inlineStr"/>
+      <c r="O58" s="4" t="inlineStr">
+        <is>
+          <t>Horse mentioned in human sample notes but no corresponding horse entry found in Horses.docx from Joe</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>Brimnes, Viðvikurhreppur</t>
+          <t>Stærri-Árskógur</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>BRV</t>
+          <t>SAE</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -3859,7 +3867,7 @@
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>Þjms.6040</t>
+          <t>Þjms. 7708-1 og 2</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
@@ -3879,15 +3887,19 @@
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>Skagafjarðarsýsla</t>
-        </is>
-      </c>
-      <c r="J59" s="4" t="inlineStr"/>
+          <t>Eyjafjarðarsýsla</t>
+        </is>
+      </c>
+      <c r="J59" s="4" t="inlineStr">
+        <is>
+          <t>Norðurland</t>
+        </is>
+      </c>
       <c r="K59" s="4" t="n">
-        <v>65.777175</v>
+        <v>65.911438</v>
       </c>
       <c r="L59" s="4" t="n">
-        <v>-19.34862</v>
+        <v>-18.357794</v>
       </c>
       <c r="M59" s="4" t="inlineStr">
         <is>
@@ -3900,14 +3912,10 @@
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>Grafargerði á Höfðaströnd</t>
-        </is>
-      </c>
-      <c r="B60" s="4" t="inlineStr">
-        <is>
-          <t>GGH</t>
-        </is>
-      </c>
+          <t>Austarihóll, Haganeshreppur</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr"/>
       <c r="C60" s="4" t="inlineStr">
         <is>
           <t>In new request</t>
@@ -3918,7 +3926,7 @@
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>11685-b</t>
+          <t>óskráð hrossabein (box found)</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
@@ -3936,45 +3944,29 @@
           <t>Settlement (870–1100 CE)</t>
         </is>
       </c>
-      <c r="I60" s="4" t="inlineStr">
-        <is>
-          <t>Skagafjarðarsýsla</t>
-        </is>
-      </c>
-      <c r="J60" s="4" t="inlineStr">
-        <is>
-          <t>Norðurland</t>
-        </is>
-      </c>
+      <c r="I60" s="4" t="inlineStr"/>
+      <c r="J60" s="4" t="inlineStr"/>
       <c r="K60" s="4" t="n">
-        <v>65.881074</v>
+        <v>65.73999999999999</v>
       </c>
       <c r="L60" s="4" t="n">
-        <v>-19.392373</v>
+        <v>-19.31</v>
       </c>
       <c r="M60" s="4" t="inlineStr">
         <is>
-          <t>ISN93→WGS84</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="N60" s="4" t="inlineStr"/>
-      <c r="O60" s="4" t="inlineStr">
-        <is>
-          <t>Horse mentioned in human sample notes but no corresponding horse entry found in Horses.docx from Joe</t>
-        </is>
-      </c>
+      <c r="O60" s="4" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>Stærri-Árskógur</t>
-        </is>
-      </c>
-      <c r="B61" s="4" t="inlineStr">
-        <is>
-          <t>SAE</t>
-        </is>
-      </c>
+          <t>Eyvindarveri</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr"/>
       <c r="C61" s="4" t="inlineStr">
         <is>
           <t>In new request</t>
@@ -3985,43 +3977,35 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 7708-1 og 2</t>
+          <t>1996-269</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>&lt; 1000</t>
+          <t>1772</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>settlement</t>
+          <t>post-settlement</t>
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t>Settlement (870–1100 CE)</t>
-        </is>
-      </c>
-      <c r="I61" s="4" t="inlineStr">
-        <is>
-          <t>Eyjafjarðarsýsla</t>
-        </is>
-      </c>
-      <c r="J61" s="4" t="inlineStr">
-        <is>
-          <t>Norðurland</t>
-        </is>
-      </c>
+          <t>Laki era (~1780 CE)</t>
+        </is>
+      </c>
+      <c r="I61" s="4" t="inlineStr"/>
+      <c r="J61" s="4" t="inlineStr"/>
       <c r="K61" s="4" t="n">
-        <v>65.911438</v>
+        <v>64.137</v>
       </c>
       <c r="L61" s="4" t="n">
-        <v>-18.357794</v>
+        <v>-18.718</v>
       </c>
       <c r="M61" s="4" t="inlineStr">
         <is>
-          <t>ISN93→WGS84</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="N61" s="4" t="inlineStr"/>
@@ -4030,7 +4014,7 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>Austarihóll, Haganeshreppur</t>
+          <t>Galtalækur/Land</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr"/>
@@ -4044,7 +4028,7 @@
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>óskráð hrossabein (box found)</t>
+          <t>Þjms. 10493</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
@@ -4065,10 +4049,10 @@
       <c r="I62" s="4" t="inlineStr"/>
       <c r="J62" s="4" t="inlineStr"/>
       <c r="K62" s="4" t="n">
-        <v>65.73999999999999</v>
+        <v>64</v>
       </c>
       <c r="L62" s="4" t="n">
-        <v>-19.31</v>
+        <v>-19.95</v>
       </c>
       <c r="M62" s="4" t="inlineStr">
         <is>
@@ -4081,7 +4065,7 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>Eyvindarveri</t>
+          <t>Grafarbakki, Rangárvallarhreppur</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr"/>
@@ -4091,39 +4075,39 @@
         </is>
       </c>
       <c r="D63" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>1996-269</t>
+          <t>hrossabein úr tveimur kumlum</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>1772</t>
+          <t>&lt; 1000</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>post-settlement</t>
+          <t>settlement</t>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr">
         <is>
-          <t>Laki era (~1780 CE)</t>
+          <t>Settlement (870–1100 CE)</t>
         </is>
       </c>
       <c r="I63" s="4" t="inlineStr"/>
       <c r="J63" s="4" t="inlineStr"/>
       <c r="K63" s="4" t="n">
-        <v>64.137</v>
+        <v>64.13424999999999</v>
       </c>
       <c r="L63" s="4" t="n">
-        <v>-18.718</v>
+        <v>-20.309083</v>
       </c>
       <c r="M63" s="4" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>DMS→WGS84</t>
         </is>
       </c>
       <c r="N63" s="4" t="inlineStr"/>
@@ -4132,7 +4116,7 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>Galtalækur/Land</t>
+          <t>Granastaðir</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr"/>
@@ -4142,11 +4126,11 @@
         </is>
       </c>
       <c r="D64" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 10493</t>
+          <t>2011-49-126 (#8); 2011-49-212 (#4); 2011-49-219 (#2); 2011-49-252 (#9)</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
@@ -4167,14 +4151,14 @@
       <c r="I64" s="4" t="inlineStr"/>
       <c r="J64" s="4" t="inlineStr"/>
       <c r="K64" s="4" t="n">
-        <v>64</v>
+        <v>65.300889</v>
       </c>
       <c r="L64" s="4" t="n">
-        <v>-19.95</v>
+        <v>-18.247528</v>
       </c>
       <c r="M64" s="4" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>DMS→WGS84</t>
         </is>
       </c>
       <c r="N64" s="4" t="inlineStr"/>
@@ -4183,7 +4167,7 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>Grafarbakki, Rangárvallarhreppur</t>
+          <t>Hafurbjarnarstaðir</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr"/>
@@ -4193,11 +4177,11 @@
         </is>
       </c>
       <c r="D65" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>hrossabein úr tveimur kumlum</t>
+          <t>Þjms. 571</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
@@ -4218,10 +4202,10 @@
       <c r="I65" s="4" t="inlineStr"/>
       <c r="J65" s="4" t="inlineStr"/>
       <c r="K65" s="4" t="n">
-        <v>64.13424999999999</v>
+        <v>64.069833</v>
       </c>
       <c r="L65" s="4" t="n">
-        <v>-20.309083</v>
+        <v>-22.700028</v>
       </c>
       <c r="M65" s="4" t="inlineStr">
         <is>
@@ -4234,7 +4218,7 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>Granastaðir</t>
+          <t>Hvalnes</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr"/>
@@ -4244,35 +4228,35 @@
         </is>
       </c>
       <c r="D66" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>2011-49-126 (#8); 2011-49-212 (#4); 2011-49-219 (#2); 2011-49-252 (#9)</t>
+          <t>Þjms. 11726</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>&lt; 1000</t>
+          <t>undated</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>settlement</t>
+          <t>undated</t>
         </is>
       </c>
       <c r="H66" s="4" t="inlineStr">
         <is>
-          <t>Settlement (870–1100 CE)</t>
+          <t>Undated</t>
         </is>
       </c>
       <c r="I66" s="4" t="inlineStr"/>
       <c r="J66" s="4" t="inlineStr"/>
       <c r="K66" s="4" t="n">
-        <v>65.300889</v>
+        <v>64.410056</v>
       </c>
       <c r="L66" s="4" t="n">
-        <v>-18.247528</v>
+        <v>-14.552306</v>
       </c>
       <c r="M66" s="4" t="inlineStr">
         <is>
@@ -4285,7 +4269,7 @@
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>Hafurbjarnarstaðir</t>
+          <t>Hörgsdalur/Mývatnsheiði</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr"/>
@@ -4299,31 +4283,31 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 571</t>
+          <t>Þjms. 4992</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>&lt; 1000</t>
+          <t>undated</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>settlement</t>
+          <t>undated</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr">
         <is>
-          <t>Settlement (870–1100 CE)</t>
+          <t>Undated</t>
         </is>
       </c>
       <c r="I67" s="4" t="inlineStr"/>
       <c r="J67" s="4" t="inlineStr"/>
       <c r="K67" s="4" t="n">
-        <v>64.069833</v>
+        <v>65.545028</v>
       </c>
       <c r="L67" s="4" t="n">
-        <v>-22.700028</v>
+        <v>-17.292861</v>
       </c>
       <c r="M67" s="4" t="inlineStr">
         <is>
@@ -4336,7 +4320,7 @@
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>Hvalnes</t>
+          <t>Kirkjubæ á Síðu</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr"/>
@@ -4350,31 +4334,31 @@
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 11726</t>
+          <t>Þjms. 13114</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>undated</t>
+          <t>&lt; 1000</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>undated</t>
+          <t>settlement</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr">
         <is>
-          <t>Undated</t>
+          <t>Settlement (870–1100 CE)</t>
         </is>
       </c>
       <c r="I68" s="4" t="inlineStr"/>
       <c r="J68" s="4" t="inlineStr"/>
       <c r="K68" s="4" t="n">
-        <v>64.410056</v>
+        <v>63.789</v>
       </c>
       <c r="L68" s="4" t="n">
-        <v>-14.552306</v>
+        <v>-18.0531</v>
       </c>
       <c r="M68" s="4" t="inlineStr">
         <is>
@@ -4387,7 +4371,7 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>Hörgsdalur/Mývatnsheiði</t>
+          <t>Litli-Dunhagi/Hörgárdal</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr"/>
@@ -4401,31 +4385,31 @@
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>Þjms. 4992</t>
+          <t>Þjms. 1963-153</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>undated</t>
+          <t>&lt; 1000</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>undated</t>
+          <t>settlement</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr">
         <is>
-          <t>Undated</t>
+          <t>Settlement (870–1100 CE)</t>
         </is>
       </c>
       <c r="I69" s="4" t="inlineStr"/>
       <c r="J69" s="4" t="inlineStr"/>
       <c r="K69" s="4" t="n">
-        <v>65.545028</v>
+        <v>65.75580600000001</v>
       </c>
       <c r="L69" s="4" t="n">
-        <v>-17.292861</v>
+        <v>-18.276556</v>
       </c>
       <c r="M69" s="4" t="inlineStr">
         <is>
@@ -4434,108 +4418,6 @@
       </c>
       <c r="N69" s="4" t="inlineStr"/>
       <c r="O69" s="4" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="4" t="inlineStr">
-        <is>
-          <t>Kirkjubæ á Síðu</t>
-        </is>
-      </c>
-      <c r="B70" s="4" t="inlineStr"/>
-      <c r="C70" s="4" t="inlineStr">
-        <is>
-          <t>In new request</t>
-        </is>
-      </c>
-      <c r="D70" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E70" s="4" t="inlineStr">
-        <is>
-          <t>Þjms. 13114</t>
-        </is>
-      </c>
-      <c r="F70" s="4" t="inlineStr">
-        <is>
-          <t>&lt; 1000</t>
-        </is>
-      </c>
-      <c r="G70" s="4" t="inlineStr">
-        <is>
-          <t>settlement</t>
-        </is>
-      </c>
-      <c r="H70" s="4" t="inlineStr">
-        <is>
-          <t>Settlement (870–1100 CE)</t>
-        </is>
-      </c>
-      <c r="I70" s="4" t="inlineStr"/>
-      <c r="J70" s="4" t="inlineStr"/>
-      <c r="K70" s="4" t="n">
-        <v>63.789</v>
-      </c>
-      <c r="L70" s="4" t="n">
-        <v>-18.0531</v>
-      </c>
-      <c r="M70" s="4" t="inlineStr">
-        <is>
-          <t>DMS→WGS84</t>
-        </is>
-      </c>
-      <c r="N70" s="4" t="inlineStr"/>
-      <c r="O70" s="4" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="4" t="inlineStr">
-        <is>
-          <t>Litli-Dunhagi/Hörgárdal</t>
-        </is>
-      </c>
-      <c r="B71" s="4" t="inlineStr"/>
-      <c r="C71" s="4" t="inlineStr">
-        <is>
-          <t>In new request</t>
-        </is>
-      </c>
-      <c r="D71" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E71" s="4" t="inlineStr">
-        <is>
-          <t>Þjms. 1963-153</t>
-        </is>
-      </c>
-      <c r="F71" s="4" t="inlineStr">
-        <is>
-          <t>&lt; 1000</t>
-        </is>
-      </c>
-      <c r="G71" s="4" t="inlineStr">
-        <is>
-          <t>settlement</t>
-        </is>
-      </c>
-      <c r="H71" s="4" t="inlineStr">
-        <is>
-          <t>Settlement (870–1100 CE)</t>
-        </is>
-      </c>
-      <c r="I71" s="4" t="inlineStr"/>
-      <c r="J71" s="4" t="inlineStr"/>
-      <c r="K71" s="4" t="n">
-        <v>65.75580600000001</v>
-      </c>
-      <c r="L71" s="4" t="n">
-        <v>-18.276556</v>
-      </c>
-      <c r="M71" s="4" t="inlineStr">
-        <is>
-          <t>DMS→WGS84</t>
-        </is>
-      </c>
-      <c r="N71" s="4" t="inlineStr"/>
-      <c r="O71" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:O71"/>

</xml_diff>

<commit_message>
Add Daðastaðir and Hofstaðir to CSV/xlsx with coordinates; update sampling request
- Daðastaðir (DAP): 65.705, -17.275, N=2, post-settlement
- Hofstaðir (HST): 65.608, -17.1638, N=1, settlement
- Sampling request: HST dyrabein row now identified as Hofstaðir

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/draftsNew/horse_sites_wgs84.xlsx
+++ b/draftsNew/horse_sites_wgs84.xlsx
@@ -36,7 +36,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +63,12 @@
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -76,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -85,6 +91,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -450,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O69"/>
+  <dimension ref="A1:O71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -4419,6 +4426,128 @@
       <c r="N69" s="4" t="inlineStr"/>
       <c r="O69" s="4" t="inlineStr"/>
     </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>Daðastaðir</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>DAP</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>In new request</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr">
+        <is>
+          <t>DAD 07 #17 (K-5-0-5); Daðastaðir 2005 K-5-D-1 and K-5-D-2</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>pre-1300</t>
+        </is>
+      </c>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>post-settlement</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>Post-medieval (1100–1900 CE)</t>
+        </is>
+      </c>
+      <c r="I70" s="6" t="inlineStr"/>
+      <c r="J70" s="6" t="inlineStr">
+        <is>
+          <t>Norðurland</t>
+        </is>
+      </c>
+      <c r="K70" s="6" t="n">
+        <v>65.705</v>
+      </c>
+      <c r="L70" s="6" t="n">
+        <v>-17.275</v>
+      </c>
+      <c r="M70" s="6" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="N70" s="6" t="inlineStr"/>
+      <c r="O70" s="6" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>Hofstaðir</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>HST</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>In new request</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="inlineStr">
+        <is>
+          <t>HST dyrabein (boxes 32, 35, 37)</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>&lt; 1000</t>
+        </is>
+      </c>
+      <c r="G71" s="6" t="inlineStr">
+        <is>
+          <t>settlement</t>
+        </is>
+      </c>
+      <c r="H71" s="6" t="inlineStr">
+        <is>
+          <t>Settlement (870–1100 CE)</t>
+        </is>
+      </c>
+      <c r="I71" s="6" t="inlineStr"/>
+      <c r="J71" s="6" t="inlineStr">
+        <is>
+          <t>Norðurland</t>
+        </is>
+      </c>
+      <c r="K71" s="6" t="n">
+        <v>65.608</v>
+      </c>
+      <c r="L71" s="6" t="n">
+        <v>-17.1638</v>
+      </c>
+      <c r="M71" s="6" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="N71" s="6" t="inlineStr"/>
+      <c r="O71" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>